<commit_message>
Diagram of sample names, with examples
</commit_message>
<xml_diff>
--- a/MINAGRIS_Plastic.R_ReadMe.xlsx
+++ b/MINAGRIS_Plastic.R_ReadMe.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\berio001\Documents\MINAGRIS_C\MINAGRIS_Microplastic_Soil_Assessmnent\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B45BA00-4512-4391-BCFF-FD57EC2A8220}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A995F3AE-9E9F-45CC-9054-07AACA89C711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A634431C-1F0B-4477-A9DD-2C46E099AE2B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{A634431C-1F0B-4477-A9DD-2C46E099AE2B}"/>
   </bookViews>
   <sheets>
     <sheet name="Scripts" sheetId="1" r:id="rId1"/>
@@ -1354,6 +1354,60 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1507375</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>-1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>557729</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>103973</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F94CF7AF-4A50-FFD6-F1AB-6B3111A01FB4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7603375" y="3782290"/>
+          <a:ext cx="12142899" cy="3886265"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2513,6 +2567,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>